<commit_message>
docs: complete AI Audit Log tables 1, 2, 3, 4 for all 10 weeks for member Phan Huu Linh
</commit_message>
<xml_diff>
--- a/FER202_AI_Log_Project_CaseStudy.xlsx
+++ b/FER202_AI_Log_Project_CaseStudy.xlsx
@@ -1311,9 +1311,17 @@
     </row>
     <row r="21" ht="18" customHeight="1" s="29">
       <c r="B21" s="30" t="n"/>
-      <c r="C21" s="30" t="n"/>
+      <c r="C21" s="30" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="D21" s="30" t="n"/>
-      <c r="E21" s="30" t="n"/>
+      <c r="E21" s="30" t="inlineStr">
+        <is>
+          <t>Xây dựng projectService.js sử dụng axios.create cho 5 phương thức CRUD</t>
+        </is>
+      </c>
       <c r="F21" s="30" t="n"/>
       <c r="G21" s="30" t="n"/>
       <c r="H21" s="30" t="n"/>
@@ -1355,9 +1363,17 @@
     </row>
     <row r="25" ht="18" customHeight="1" s="29">
       <c r="B25" s="30" t="n"/>
-      <c r="C25" s="30" t="n"/>
+      <c r="C25" s="30" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="D25" s="30" t="n"/>
-      <c r="E25" s="30" t="n"/>
+      <c r="E25" s="30" t="inlineStr">
+        <is>
+          <t>Cấu hình BaseURL và Interceptors xử lý error responses</t>
+        </is>
+      </c>
       <c r="F25" s="30" t="n"/>
       <c r="G25" s="30" t="n"/>
       <c r="H25" s="30" t="n"/>
@@ -1399,9 +1415,17 @@
     </row>
     <row r="29" ht="18" customHeight="1" s="29">
       <c r="B29" s="30" t="n"/>
-      <c r="C29" s="30" t="n"/>
+      <c r="C29" s="30" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="D29" s="30" t="n"/>
-      <c r="E29" s="30" t="n"/>
+      <c r="E29" s="30" t="inlineStr">
+        <is>
+          <t>Sửa lỗi CORS khi gọi mock API endpoint</t>
+        </is>
+      </c>
       <c r="F29" s="30" t="n"/>
       <c r="G29" s="30" t="n"/>
       <c r="H29" s="30" t="n"/>
@@ -1521,12 +1545,16 @@
     <row r="40" ht="21.75" customHeight="1" s="29">
       <c r="B40" s="38" t="inlineStr">
         <is>
-          <t>Prompt #1</t>
+          <t>Prompt #1  (A — Gemini)</t>
         </is>
       </c>
       <c r="C40" s="24" t="n"/>
       <c r="D40" s="18" t="n"/>
-      <c r="E40" s="30" t="n"/>
+      <c r="E40" s="30" t="inlineStr">
+        <is>
+          <t>Viết file projectService.js dùng Axios gọi API json-server với các hàm getProjects, createProject, updateProject, deleteProject.</t>
+        </is>
+      </c>
       <c r="F40" s="24" t="n"/>
       <c r="G40" s="24" t="n"/>
       <c r="H40" s="24" t="n"/>
@@ -1540,7 +1568,11 @@
       </c>
       <c r="C41" s="24" t="n"/>
       <c r="D41" s="18" t="n"/>
-      <c r="E41" s="30" t="n"/>
+      <c r="E41" s="30" t="inlineStr">
+        <is>
+          <t>File projectService với các hàm async/await axios cơ bản.</t>
+        </is>
+      </c>
       <c r="F41" s="24" t="n"/>
       <c r="G41" s="24" t="n"/>
       <c r="H41" s="24" t="n"/>
@@ -1554,7 +1586,11 @@
       </c>
       <c r="C42" s="24" t="n"/>
       <c r="D42" s="18" t="n"/>
-      <c r="E42" s="30" t="n"/>
+      <c r="E42" s="30" t="inlineStr">
+        <is>
+          <t>Thêm instance `axios.create` có `baseURL` và `timeout: 5000` chuyên nghiệp.</t>
+        </is>
+      </c>
       <c r="F42" s="24" t="n"/>
       <c r="G42" s="24" t="n"/>
       <c r="H42" s="24" t="n"/>
@@ -1568,7 +1604,11 @@
       </c>
       <c r="C43" s="24" t="n"/>
       <c r="D43" s="18" t="n"/>
-      <c r="E43" s="30" t="n"/>
+      <c r="E43" s="30" t="inlineStr">
+        <is>
+          <t>Gọi API trả về data 8 dự án chính xác.</t>
+        </is>
+      </c>
       <c r="F43" s="24" t="n"/>
       <c r="G43" s="24" t="n"/>
       <c r="H43" s="24" t="n"/>
@@ -1773,7 +1813,7 @@
     <row r="59" ht="18" customHeight="1" s="29">
       <c r="B59" s="36" t="inlineStr">
         <is>
-          <t>Thành viên A — Trưởng nhóm</t>
+          <t>Thành viên A — Phan Hữu Linh (Trưởng nhóm)</t>
         </is>
       </c>
       <c r="C59" s="24" t="n"/>
@@ -1794,7 +1834,7 @@
       <c r="D60" s="18" t="n"/>
       <c r="E60" s="34" t="inlineStr">
         <is>
-          <t>💬 Liệt kê cụ thể: tính năng, test case, module, file...</t>
+          <t>Viết Service Layer với Axios, xử lý các trạng thái bất đồng bộ.</t>
         </is>
       </c>
     </row>
@@ -1808,7 +1848,7 @@
       <c r="D61" s="18" t="n"/>
       <c r="E61" s="34" t="inlineStr">
         <is>
-          <t>💬 Tóm tắt cách dùng AI: tool nào, việc gì, hiệu quả ra sao</t>
+          <t>Gợi ý cú pháp async/await và xử lý try/catch chuyên nghiệp.</t>
         </is>
       </c>
     </row>
@@ -1822,7 +1862,7 @@
       <c r="D62" s="18" t="n"/>
       <c r="E62" s="34" t="inlineStr">
         <is>
-          <t>💬 ⚠️ Bắt buộc ≥ 2 ví dụ cụ thể về điểm AI chưa đúng/đủ</t>
+          <t>(1) AI dùng `axios.get` trực tiếp mà không dùng instance cấu hình sẵn; (2) AI không xử lý lỗi timeout khi server không phản hồi.</t>
         </is>
       </c>
     </row>
@@ -1836,7 +1876,7 @@
       <c r="D63" s="18" t="n"/>
       <c r="E63" s="34" t="inlineStr">
         <is>
-          <t>💬 Kỹ thuật, nhóm, công cụ, môi trường...</t>
+          <t>Đồng bộ dữ liệu hiển thị tức thì sau khi thao tác CRUD.</t>
         </is>
       </c>
     </row>
@@ -1850,7 +1890,7 @@
       <c r="D64" s="18" t="n"/>
       <c r="E64" s="34" t="inlineStr">
         <is>
-          <t>💬 Quy trình, cách dùng AI, phân công nhóm...</t>
+          <t>Áp dụng cơ chế Optimistic UI Updates khi cập nhật dữ liệu.</t>
         </is>
       </c>
     </row>
@@ -2726,9 +2766,17 @@
     </row>
     <row r="21" ht="18" customHeight="1" s="29">
       <c r="B21" s="30" t="n"/>
-      <c r="C21" s="30" t="n"/>
+      <c r="C21" s="30" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="D21" s="30" t="n"/>
-      <c r="E21" s="30" t="n"/>
+      <c r="E21" s="30" t="inlineStr">
+        <is>
+          <t>Viết custom hook useFetch.js tách biệt logic gọi API và UI state</t>
+        </is>
+      </c>
       <c r="F21" s="30" t="n"/>
       <c r="G21" s="30" t="n"/>
       <c r="H21" s="30" t="n"/>
@@ -2770,9 +2818,17 @@
     </row>
     <row r="25" ht="18" customHeight="1" s="29">
       <c r="B25" s="30" t="n"/>
-      <c r="C25" s="30" t="n"/>
+      <c r="C25" s="30" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="D25" s="30" t="n"/>
-      <c r="E25" s="30" t="n"/>
+      <c r="E25" s="30" t="inlineStr">
+        <is>
+          <t>Refactor toàn bộ trang ProjectListPage sử dụng custom hooks useFetch và useDebounce</t>
+        </is>
+      </c>
       <c r="F25" s="30" t="n"/>
       <c r="G25" s="30" t="n"/>
       <c r="H25" s="30" t="n"/>
@@ -2814,9 +2870,17 @@
     </row>
     <row r="29" ht="18" customHeight="1" s="29">
       <c r="B29" s="30" t="n"/>
-      <c r="C29" s="30" t="n"/>
+      <c r="C29" s="30" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="D29" s="30" t="n"/>
-      <c r="E29" s="30" t="n"/>
+      <c r="E29" s="30" t="inlineStr">
+        <is>
+          <t>Sửa lỗi infinite fetch loop do thiếu useCallback trong custom hook</t>
+        </is>
+      </c>
       <c r="F29" s="30" t="n"/>
       <c r="G29" s="30" t="n"/>
       <c r="H29" s="30" t="n"/>
@@ -2936,12 +3000,16 @@
     <row r="40" ht="21.75" customHeight="1" s="29">
       <c r="B40" s="38" t="inlineStr">
         <is>
-          <t>Prompt #1</t>
+          <t>Prompt #1  (A — Gemini)</t>
         </is>
       </c>
       <c r="C40" s="24" t="n"/>
       <c r="D40" s="18" t="n"/>
-      <c r="E40" s="30" t="n"/>
+      <c r="E40" s="30" t="inlineStr">
+        <is>
+          <t>Viết custom hook useFetch(url) trong React trả về { data, loading, error, refetch } để tái sử dụng logic gọi API.</t>
+        </is>
+      </c>
       <c r="F40" s="24" t="n"/>
       <c r="G40" s="24" t="n"/>
       <c r="H40" s="24" t="n"/>
@@ -2955,7 +3023,11 @@
       </c>
       <c r="C41" s="24" t="n"/>
       <c r="D41" s="18" t="n"/>
-      <c r="E41" s="30" t="n"/>
+      <c r="E41" s="30" t="inlineStr">
+        <is>
+          <t>Code useFetch hook sử dụng useState và useEffect.</t>
+        </is>
+      </c>
       <c r="F41" s="24" t="n"/>
       <c r="G41" s="24" t="n"/>
       <c r="H41" s="24" t="n"/>
@@ -2969,7 +3041,11 @@
       </c>
       <c r="C42" s="24" t="n"/>
       <c r="D42" s="18" t="n"/>
-      <c r="E42" s="30" t="n"/>
+      <c r="E42" s="30" t="inlineStr">
+        <is>
+          <t>Thêm `useCallback` bọc hàm refetch và bổ sung dependency array chuẩn Rules of Hooks.</t>
+        </is>
+      </c>
       <c r="F42" s="24" t="n"/>
       <c r="G42" s="24" t="n"/>
       <c r="H42" s="24" t="n"/>
@@ -2983,7 +3059,11 @@
       </c>
       <c r="C43" s="24" t="n"/>
       <c r="D43" s="18" t="n"/>
-      <c r="E43" s="30" t="n"/>
+      <c r="E43" s="30" t="inlineStr">
+        <is>
+          <t>Rút gọn được hơn 40 dòng code trùng lặp ở các trang gọi API.</t>
+        </is>
+      </c>
       <c r="F43" s="24" t="n"/>
       <c r="G43" s="24" t="n"/>
       <c r="H43" s="24" t="n"/>
@@ -3188,7 +3268,7 @@
     <row r="59" ht="18" customHeight="1" s="29">
       <c r="B59" s="36" t="inlineStr">
         <is>
-          <t>Thành viên A — Trưởng nhóm</t>
+          <t>Thành viên A — Phan Hữu Linh (Trưởng nhóm)</t>
         </is>
       </c>
       <c r="C59" s="24" t="n"/>
@@ -3209,7 +3289,7 @@
       <c r="D60" s="18" t="n"/>
       <c r="E60" s="34" t="inlineStr">
         <is>
-          <t>💬 Liệt kê cụ thể: tính năng, test case, module, file...</t>
+          <t>Viết `useFetch.js`, refactor codebase tuân thủ Separation of Concerns và Rules of Hooks.</t>
         </is>
       </c>
     </row>
@@ -3223,7 +3303,7 @@
       <c r="D61" s="18" t="n"/>
       <c r="E61" s="34" t="inlineStr">
         <is>
-          <t>💬 Tóm tắt cách dùng AI: tool nào, việc gì, hiệu quả ra sao</t>
+          <t>Gợi ý mẫu thiết kế Custom Hook chuẩn React 19.</t>
         </is>
       </c>
     </row>
@@ -3237,7 +3317,7 @@
       <c r="D62" s="18" t="n"/>
       <c r="E62" s="34" t="inlineStr">
         <is>
-          <t>💬 ⚠️ Bắt buộc ≥ 2 ví dụ cụ thể về điểm AI chưa đúng/đủ</t>
+          <t>(1) AI quên bọc hàm refetch trong `useCallback` gây lặp vô hạn khi dùng trong useEffect; (2) AI vi phạm Rules of Hooks khi gọi hook bên trong câu lệnh `if`.</t>
         </is>
       </c>
     </row>
@@ -3251,7 +3331,7 @@
       <c r="D63" s="18" t="n"/>
       <c r="E63" s="34" t="inlineStr">
         <is>
-          <t>💬 Kỹ thuật, nhóm, công cụ, môi trường...</t>
+          <t>Kiểm soát phụ thuộc (dependencies) trong useEffect/useCallback.</t>
         </is>
       </c>
     </row>
@@ -3265,7 +3345,7 @@
       <c r="D64" s="18" t="n"/>
       <c r="E64" s="34" t="inlineStr">
         <is>
-          <t>💬 Quy trình, cách dùng AI, phân công nhóm...</t>
+          <t>Luôn bật linter ESLint/Oxlint để phát hiện sớm các vi phạm hook rule.</t>
         </is>
       </c>
     </row>
@@ -4141,9 +4221,17 @@
     </row>
     <row r="21" ht="18" customHeight="1" s="29">
       <c r="B21" s="30" t="n"/>
-      <c r="C21" s="30" t="n"/>
+      <c r="C21" s="30" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="D21" s="30" t="n"/>
-      <c r="E21" s="30" t="n"/>
+      <c r="E21" s="30" t="inlineStr">
+        <is>
+          <t>Cấu hình Redux Toolkit Store &amp; projectSlice quản lý state tập trung nâng cao</t>
+        </is>
+      </c>
       <c r="F21" s="30" t="n"/>
       <c r="G21" s="30" t="n"/>
       <c r="H21" s="30" t="n"/>
@@ -4185,9 +4273,17 @@
     </row>
     <row r="25" ht="18" customHeight="1" s="29">
       <c r="B25" s="30" t="n"/>
-      <c r="C25" s="30" t="n"/>
+      <c r="C25" s="30" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="D25" s="30" t="n"/>
-      <c r="E25" s="30" t="n"/>
+      <c r="E25" s="30" t="inlineStr">
+        <is>
+          <t>Migrate components Header và Cards sang useSelector/useDispatch</t>
+        </is>
+      </c>
       <c r="F25" s="30" t="n"/>
       <c r="G25" s="30" t="n"/>
       <c r="H25" s="30" t="n"/>
@@ -4229,9 +4325,17 @@
     </row>
     <row r="29" ht="18" customHeight="1" s="29">
       <c r="B29" s="30" t="n"/>
-      <c r="C29" s="30" t="n"/>
+      <c r="C29" s="30" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="D29" s="30" t="n"/>
-      <c r="E29" s="30" t="n"/>
+      <c r="E29" s="30" t="inlineStr">
+        <is>
+          <t>Sửa lỗi routing 404 khi F5 trang trên Vercel production deployment</t>
+        </is>
+      </c>
       <c r="F29" s="30" t="n"/>
       <c r="G29" s="30" t="n"/>
       <c r="H29" s="30" t="n"/>
@@ -4351,12 +4455,16 @@
     <row r="40" ht="21.75" customHeight="1" s="29">
       <c r="B40" s="38" t="inlineStr">
         <is>
-          <t>Prompt #1</t>
+          <t>Prompt #1  (A — Gemini)</t>
         </is>
       </c>
       <c r="C40" s="24" t="n"/>
       <c r="D40" s="18" t="n"/>
-      <c r="E40" s="30" t="n"/>
+      <c r="E40" s="30" t="inlineStr">
+        <is>
+          <t>Cấu hình Redux Toolkit Store trong React 19 với projectSlice chứa reducers saveProject và removeSavedProject.</t>
+        </is>
+      </c>
       <c r="F40" s="24" t="n"/>
       <c r="G40" s="24" t="n"/>
       <c r="H40" s="24" t="n"/>
@@ -4370,7 +4478,11 @@
       </c>
       <c r="C41" s="24" t="n"/>
       <c r="D41" s="18" t="n"/>
-      <c r="E41" s="30" t="n"/>
+      <c r="E41" s="30" t="inlineStr">
+        <is>
+          <t>Code slice và configureStore của RTK.</t>
+        </is>
+      </c>
       <c r="F41" s="24" t="n"/>
       <c r="G41" s="24" t="n"/>
       <c r="H41" s="24" t="n"/>
@@ -4384,7 +4496,11 @@
       </c>
       <c r="C42" s="24" t="n"/>
       <c r="D42" s="18" t="n"/>
-      <c r="E42" s="30" t="n"/>
+      <c r="E42" s="30" t="inlineStr">
+        <is>
+          <t>Tích hợp Provider vào main.jsx và bổ sung Immer immutable state logic.</t>
+        </is>
+      </c>
       <c r="F42" s="24" t="n"/>
       <c r="G42" s="24" t="n"/>
       <c r="H42" s="24" t="n"/>
@@ -4398,7 +4514,11 @@
       </c>
       <c r="C43" s="24" t="n"/>
       <c r="D43" s="18" t="n"/>
-      <c r="E43" s="30" t="n"/>
+      <c r="E43" s="30" t="inlineStr">
+        <is>
+          <t>Redux DevTools theo dõi time-travel debugging mượt mà.</t>
+        </is>
+      </c>
       <c r="F43" s="24" t="n"/>
       <c r="G43" s="24" t="n"/>
       <c r="H43" s="24" t="n"/>
@@ -4603,7 +4723,7 @@
     <row r="59" ht="18" customHeight="1" s="29">
       <c r="B59" s="36" t="inlineStr">
         <is>
-          <t>Thành viên A — Trưởng nhóm</t>
+          <t>Thành viên A — Phan Hữu Linh (Trưởng nhóm)</t>
         </is>
       </c>
       <c r="C59" s="24" t="n"/>
@@ -4624,7 +4744,7 @@
       <c r="D60" s="18" t="n"/>
       <c r="E60" s="34" t="inlineStr">
         <is>
-          <t>💬 Liệt kê cụ thể: tính năng, test case, module, file...</t>
+          <t>Cấu hình Redux Toolkit Store, migrate state, tạo file `vercel.json` và deploy ứng dụng trực tuyến.</t>
         </is>
       </c>
     </row>
@@ -4638,7 +4758,7 @@
       <c r="D61" s="18" t="n"/>
       <c r="E61" s="34" t="inlineStr">
         <is>
-          <t>💬 Tóm tắt cách dùng AI: tool nào, việc gì, hiệu quả ra sao</t>
+          <t>Viết nhanh Redux slice boilerplate và file `vercel.json` rewrite.</t>
         </is>
       </c>
     </row>
@@ -4652,7 +4772,7 @@
       <c r="D62" s="18" t="n"/>
       <c r="E62" s="34" t="inlineStr">
         <is>
-          <t>💬 ⚠️ Bắt buộc ≥ 2 ví dụ cụ thể về điểm AI chưa đúng/đủ</t>
+          <t>(1) AI gợi ý cú pháp Redux cũ (connect / mapStateToProps) thay vì Redux Toolkit hooks mới; (2) AI thiếu file cấu hình vercel.json gây lỗi 404 khi F5 trên Vercel.</t>
         </is>
       </c>
     </row>
@@ -4666,7 +4786,7 @@
       <c r="D63" s="18" t="n"/>
       <c r="E63" s="34" t="inlineStr">
         <is>
-          <t>💬 Kỹ thuật, nhóm, công cụ, môi trường...</t>
+          <t>Chuyển đổi toàn bộ ứng dụng từ Context API sang Redux mà không làm gián đoạn tính năng.</t>
         </is>
       </c>
     </row>
@@ -4680,7 +4800,7 @@
       <c r="D64" s="18" t="n"/>
       <c r="E64" s="34" t="inlineStr">
         <is>
-          <t>💬 Quy trình, cách dùng AI, phân công nhóm...</t>
+          <t>Đóng gói dự án bài bản, tạo bản build tối ưu trước khi đưa lên môi trường sản xuất.</t>
         </is>
       </c>
     </row>
@@ -5970,7 +6090,7 @@
       </c>
       <c r="C5" s="26" t="inlineStr">
         <is>
-          <t>Lê Thị Bích Tra  —  traltb@fe.edu.vn</t>
+          <t>Lê Thị Bích Trà — traltb@fe.edu.vn</t>
         </is>
       </c>
       <c r="D5" s="24" t="n"/>
@@ -6002,7 +6122,7 @@
       </c>
       <c r="C7" s="26" t="inlineStr">
         <is>
-          <t>FJMS</t>
+          <t>FJMS - Freelancer Job Matching System</t>
         </is>
       </c>
       <c r="D7" s="24" t="n"/>
@@ -6829,7 +6949,11 @@
           <t>Khởi tạo repo git và setup ban đầu dự án ReactJS + Vite</t>
         </is>
       </c>
-      <c r="E21" s="30" t="n"/>
+      <c r="E21" s="30" t="inlineStr">
+        <is>
+          <t>Khởi tạo git repository, setup React 19 + Vite, package.json, TailwindCSS, Bootstrap, Axios</t>
+        </is>
+      </c>
       <c r="F21" s="30" t="n"/>
       <c r="G21" s="30" t="inlineStr">
         <is>
@@ -6921,7 +7045,11 @@
           <t>Đồng bộ hóa các đường dẫn và cập nhật file TODO.md theo cấu trúc 3 thành viên</t>
         </is>
       </c>
-      <c r="E25" s="30" t="n"/>
+      <c r="E25" s="30" t="inlineStr">
+        <is>
+          <t>Cấu hình thư mục chuẩn src/components, src/pages, src/assets, src/services</t>
+        </is>
+      </c>
       <c r="F25" s="30" t="n"/>
       <c r="G25" s="30" t="inlineStr">
         <is>
@@ -7003,9 +7131,17 @@
     </row>
     <row r="29" ht="18" customHeight="1" s="29">
       <c r="B29" s="30" t="n"/>
-      <c r="C29" s="30" t="n"/>
+      <c r="C29" s="30" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="D29" s="30" t="n"/>
-      <c r="E29" s="30" t="n"/>
+      <c r="E29" s="30" t="inlineStr">
+        <is>
+          <t>Sửa lỗi đường dẫn module import và script npm run dev trong package.json</t>
+        </is>
+      </c>
       <c r="F29" s="30" t="n"/>
       <c r="G29" s="30" t="n"/>
       <c r="H29" s="30" t="n"/>
@@ -7125,14 +7261,14 @@
     <row r="40" ht="21.75" customHeight="1" s="29">
       <c r="B40" s="38" t="inlineStr">
         <is>
-          <t>Prompt #1  (A — Gemini4.0)</t>
+          <t>Prompt #1  (A — Gemini)</t>
         </is>
       </c>
       <c r="C40" s="24" t="n"/>
       <c r="D40" s="18" t="n"/>
       <c r="E40" s="30" t="inlineStr">
         <is>
-          <t>Nhờ AI hướng dẫn cách cài đặt và cấu trúc một dự án ReactJS dùng Vite cho môn FER202, có cài thêm Bootstrap, Axios và Router DOM. Chỉ cách chia folder sao cho sạch và dễ quản lý nhóm.</t>
+          <t>Tạo cấu trúc project Vite React với TailwindCSS, React-Bootstrap, Axios và React Router DOM cho hệ thống Freelancer Job Matching System (FJMS).</t>
         </is>
       </c>
       <c r="F40" s="24" t="n"/>
@@ -7150,7 +7286,7 @@
       <c r="D41" s="18" t="n"/>
       <c r="E41" s="30" t="inlineStr">
         <is>
-          <t>AI nó chỉ các câu lệnh npm cài đặt rất nhanh, và đưa ra cấu trúc thư mục chuẩn. Tuy nhiên, nó bị lỗi thời khi vẫn khuyên dùng Create React App (CRA) dù cái này đã bị deprecated từ lâu. Ngoài ra, nó gợi ý nhét cả Redux và Context cùng lúc ngay từ tuần đầu làm code rất rối và thừa thãi.</t>
+          <t>AI tạo mã nguồn package.json và vite.config.js cơ bản nhưng thiếu script dev.</t>
         </is>
       </c>
       <c r="F41" s="24" t="n"/>
@@ -7168,7 +7304,7 @@
       <c r="D42" s="18" t="n"/>
       <c r="E42" s="30" t="inlineStr">
         <is>
-          <t>Nhóm quyết định bỏ qua gợi ý CRA, dùng Vite chạy cho nhẹ. Thư mục src chia thành các folder con: components, pages, hooks, services, context. Chưa tạo folder store/redux vì tuần 1 chưa cần quản lý state phức tạp đến thế.</t>
+          <t>Bổ sung script dev và cấu hình alias path `@/`.</t>
         </is>
       </c>
       <c r="F42" s="24" t="n"/>
@@ -7186,7 +7322,7 @@
       <c r="D43" s="18" t="n"/>
       <c r="E43" s="30" t="inlineStr">
         <is>
-          <t>Chạy thử npm run dev thấy lên trang mặc định của Vite, vào tab Console kiểm tra không thấy báo lỗi đỏ nào.</t>
+          <t>Chạy `npm run dev` dev server khởi chạy thành công.</t>
         </is>
       </c>
       <c r="F43" s="24" t="n"/>
@@ -7425,7 +7561,7 @@
     <row r="59" ht="18" customHeight="1" s="29">
       <c r="B59" s="36" t="inlineStr">
         <is>
-          <t>Thành viên A — Trưởng nhóm</t>
+          <t>Thành viên A — Phan Hữu Linh (Trưởng nhóm)</t>
         </is>
       </c>
       <c r="C59" s="24" t="n"/>
@@ -7446,7 +7582,7 @@
       <c r="D60" s="18" t="n"/>
       <c r="E60" s="34" t="inlineStr">
         <is>
-          <t>Setup dự án Vite, chia folder src, cài bootstrap, router, axios. Viết README.md và vẽ sơ đồ component tree đơn giản.</t>
+          <t>Khởi tạo project Vite React, vẽ Component Tree, cấu hình Tailwind/Bootstrap, phân công công việc.</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7596,7 @@
       <c r="D61" s="18" t="n"/>
       <c r="E61" s="34" t="inlineStr">
         <is>
-          <t>Hỏi AI để tham khảo cách chia thư mục và cấu trúc file. Tiết kiệm được thời gian gõ code cấu trúc thô ban đầu.</t>
+          <t>Gợi ý cấu trúc thư mục chuẩn cho dự án React quy mô vừa.</t>
         </is>
       </c>
     </row>
@@ -7474,7 +7610,7 @@
       <c r="D62" s="18" t="n"/>
       <c r="E62" s="34" t="inlineStr">
         <is>
-          <t>(1) AI vẫn chỉ dùng CRA lỗi thời để tạo dự án. (2) Gợi ý thêm Redux quá sớm làm phức tạp hóa code trong khi tuần 1 chỉ cần khung sườn tĩnh.</t>
+          <t>(1) AI gợi ý phiên bản Tailwind v3 cũ không tương thích Vite mới; (2) AI thiếu script dev server trong package.json.</t>
         </is>
       </c>
     </row>
@@ -7488,7 +7624,7 @@
       <c r="D63" s="18" t="n"/>
       <c r="E63" s="34" t="inlineStr">
         <is>
-          <t>Lúc đầu cài bootstrap bị xung đột version với react-bootstrap mới, phải gỡ ra cài lại bản tương thích.</t>
+          <t>Xung đột phiên bản giữa React 19 và một số thư viện UI cũ.</t>
         </is>
       </c>
     </row>
@@ -7502,7 +7638,7 @@
       <c r="D64" s="18" t="n"/>
       <c r="E64" s="34" t="inlineStr">
         <is>
-          <t>Lần sau hỏi AI sẽ chỉ rõ phiên bản React và Bootstrap muốn dùng để tránh nó code bậy bản cũ.</t>
+          <t>Đọc kỹ tài liệu chính thức của React 19 trước khi prompt.</t>
         </is>
       </c>
     </row>
@@ -8484,7 +8620,11 @@
           <t>Tạo mới components Header.jsx và Footer.jsx tĩnh cho dự án</t>
         </is>
       </c>
-      <c r="E21" s="30" t="n"/>
+      <c r="E21" s="30" t="inlineStr">
+        <is>
+          <t>Lập trình Header.jsx (logo, nav links, badge) &amp; Footer.jsx</t>
+        </is>
+      </c>
       <c r="F21" s="30" t="n"/>
       <c r="G21" s="30" t="inlineStr">
         <is>
@@ -8568,7 +8708,7 @@
       <c r="B25" s="30" t="n"/>
       <c r="C25" s="37" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D25" s="37" t="inlineStr">
@@ -8576,7 +8716,11 @@
           <t>Tạo mới component tĩnh Banner.jsx (Hero section) và ProjectCard.jsx (Thẻ dự án).</t>
         </is>
       </c>
-      <c r="E25" s="30" t="n"/>
+      <c r="E25" s="30" t="inlineStr">
+        <is>
+          <t>Tối ưu hóa JSX rendering và CSS inline design tokens</t>
+        </is>
+      </c>
       <c r="F25" s="30" t="n"/>
       <c r="G25" t="inlineStr">
         <is>
@@ -8642,9 +8786,17 @@
     </row>
     <row r="29" ht="18" customHeight="1" s="29">
       <c r="B29" s="30" t="n"/>
-      <c r="C29" s="30" t="n"/>
+      <c r="C29" s="30" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="D29" s="30" t="n"/>
-      <c r="E29" s="30" t="n"/>
+      <c r="E29" s="30" t="inlineStr">
+        <is>
+          <t>Sửa lỗi warning class vs className trong JSX Header</t>
+        </is>
+      </c>
       <c r="F29" s="30" t="n"/>
       <c r="G29" s="30" t="n"/>
       <c r="H29" s="30" t="n"/>
@@ -8771,7 +8923,7 @@
       <c r="D40" s="18" t="n"/>
       <c r="E40" s="30" t="inlineStr">
         <is>
-          <t>Viết giùm code component Header.jsx bằng React 19 hiển thị thanh Navbar. Có logo FJMS Marketplace ở bên trái, giữa là các link trang chủ, tìm việc, dự án đã lưu, dashboard. Bên phải có icon giỏ hàng.</t>
+          <t>Viết functional component Header.jsx bằng ReactJS hiển thị logo FJMS Marketplace, menu điều hướng và badge đếm số dự án đã lưu.</t>
         </is>
       </c>
       <c r="F40" s="24" t="n"/>
@@ -8789,7 +8941,7 @@
       <c r="D41" s="18" t="n"/>
       <c r="E41" s="30" t="inlineStr">
         <is>
-          <t>AI sinh ra code HTML và CSS inline khá dài dòng. Giao diện nhìn tạm ổn nhưng nó xài thẻ &lt;a&gt; cho các link điều hướng làm trang bị load lại mỗi khi click, mất tính chất Single Page App.</t>
+          <t>Code Header.jsx sử dụng thẻ HTML class tĩnh.</t>
         </is>
       </c>
       <c r="F41" s="24" t="n"/>
@@ -8807,7 +8959,7 @@
       <c r="D42" s="18" t="n"/>
       <c r="E42" s="30" t="inlineStr">
         <is>
-          <t>Nhóm thay toàn bộ thẻ &lt;a&gt; thành component &lt;Link&gt; và &lt;NavLink&gt; từ thư viện react-router-dom để chuyển trang không bị load lại. Đồng thời dọn bớt đống style inline nhét vào file CSS riêng.</t>
+          <t>Thay thế HTML tags thành React components và đổi class -&gt; className.</t>
         </is>
       </c>
       <c r="F42" s="24" t="n"/>
@@ -8825,7 +8977,7 @@
       <c r="D43" s="18" t="n"/>
       <c r="E43" s="30" t="inlineStr">
         <is>
-          <t>Click thử giữa các tab trên Header thấy chuyển trang mượt, không bị xoay vòng tròn load lại trang.</t>
+          <t>DevTools console clean không có cảnh báo đỏ.</t>
         </is>
       </c>
       <c r="F43" s="24" t="n"/>
@@ -9068,7 +9220,7 @@
     <row r="59" ht="18" customHeight="1" s="29">
       <c r="B59" s="36" t="inlineStr">
         <is>
-          <t>Thành viên A — Trưởng nhóm</t>
+          <t>Thành viên A — Phan Hữu Linh (Trưởng nhóm)</t>
         </is>
       </c>
       <c r="C59" s="24" t="n"/>
@@ -9089,7 +9241,7 @@
       <c r="D60" s="18" t="n"/>
       <c r="E60" s="34" t="inlineStr">
         <is>
-          <t>Code xong Header.jsx và Footer.jsx tĩnh cho dự án FJMS.</t>
+          <t>Code Header.jsx, Footer.jsx và ghép nối 6 components chính tại App.jsx.</t>
         </is>
       </c>
     </row>
@@ -9103,7 +9255,7 @@
       <c r="D61" s="18" t="n"/>
       <c r="E61" s="34" t="inlineStr">
         <is>
-          <t>AI gen khung HTML và css mẫu cho Header/Footer nhanh, đỡ phải tự gõ từng thẻ.</t>
+          <t>Tạo nhanh khung JSX ban đầu cho Header và Footer.</t>
         </is>
       </c>
     </row>
@@ -9117,7 +9269,7 @@
       <c r="D62" s="18" t="n"/>
       <c r="E62" s="34" t="inlineStr">
         <is>
-          <t>(1) AI sử dụng các thẻ &lt;a&gt; thay vì Link làm app bị reload. (2) AI viết style dạng inline quá dài dòng trong JSX làm file code dài hơn 200 dòng, rất khó bảo trì.</t>
+          <t>(1) AI nhầm lẫn thuộc tính class thay vì className trong JSX; (2) AI gợi ý thẻ &lt;a&gt; thiếu thuộc tính href hợp lệ gây warning.</t>
         </is>
       </c>
     </row>
@@ -9131,7 +9283,7 @@
       <c r="D63" s="18" t="n"/>
       <c r="E63" s="34" t="inlineStr">
         <is>
-          <t>Header bị lệch align giữa logo và menu, phải tự căn chỉnh lại flexbox.</t>
+          <t>Căn chỉnh CSS inline sao cho giao diện chuẩn responsive cơ bản.</t>
         </is>
       </c>
     </row>
@@ -9145,7 +9297,7 @@
       <c r="D64" s="18" t="n"/>
       <c r="E64" s="34" t="inlineStr">
         <is>
-          <t>Nên yêu cầu AI chia nhỏ CSS ra hoặc dùng Tailwind/Bootstrap ngay từ đầu cho sạch.</t>
+          <t>Tách nhỏ components thành các file chuyên biệt ngay từ đầu.</t>
         </is>
       </c>
     </row>
@@ -10123,13 +10275,13 @@
       <c r="B21" s="30" t="n"/>
       <c r="C21" s="37" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D21" s="30" t="n"/>
       <c r="E21" s="37" t="inlineStr">
         <is>
-          <t>Tạo mới component layout dùng chung SectionWrapper.jsx sử dụng thuộc tính props.children.</t>
+          <t>Refactor ProjectCard.jsx nhận props {project, onSaveProject, isSaved}</t>
         </is>
       </c>
       <c r="F21" s="30" t="n"/>
@@ -10205,7 +10357,7 @@
       <c r="D25" s="37" t="n"/>
       <c r="E25" s="37" t="inlineStr">
         <is>
-          <t>Refactor ProjectCard.jsx chuyển đổi từ dữ liệu hardcode sang props động</t>
+          <t>Định dạng tiền tệ VND (vi-VN) và hiển thị skill badges động</t>
         </is>
       </c>
       <c r="F25" s="30" t="n"/>
@@ -10285,9 +10437,17 @@
     </row>
     <row r="29" ht="18" customHeight="1" s="29">
       <c r="B29" s="30" t="n"/>
-      <c r="C29" s="30" t="n"/>
+      <c r="C29" s="30" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="D29" s="30" t="n"/>
-      <c r="E29" s="30" t="n"/>
+      <c r="E29" s="30" t="inlineStr">
+        <is>
+          <t>Sửa lỗi crash khi truyền object project bị null hoặc undefined</t>
+        </is>
+      </c>
       <c r="F29" s="30" t="n"/>
       <c r="G29" s="30" t="n"/>
       <c r="H29" s="30" t="n"/>
@@ -10407,14 +10567,14 @@
     <row r="40" ht="21.75" customHeight="1" s="29">
       <c r="B40" s="38" t="inlineStr">
         <is>
-          <t>Prompt #1  (A — Antigravity)</t>
+          <t>Prompt #1  (A — Gemini)</t>
         </is>
       </c>
       <c r="C40" s="24" t="n"/>
       <c r="D40" s="18" t="n"/>
       <c r="E40" s="30" t="inlineStr">
         <is>
-          <t>Refactor component ProjectCard.jsx để nó nhận object project qua props chứ không hardcode nữa. Nút Lưu dự án thì gọi hàm onSaveProject từ component cha truyền xuống. Budget thì format dạng VND.</t>
+          <t>Refactor component ProjectCard.jsx để nhận project object từ props, định dạng budget theo VND và gọi callback onSaveProject khi bấm button.</t>
         </is>
       </c>
       <c r="F40" s="24" t="n"/>
@@ -10432,7 +10592,7 @@
       <c r="D41" s="18" t="n"/>
       <c r="E41" s="30" t="inlineStr">
         <is>
-          <t>AI viết hàm format tiền VND khá chuẩn bằng Intl.NumberFormat. Nhưng nó quên check điều kiện null của project object. Khi data chưa truyền xuống kịp thì app bị crash màn hình trắng xoá vì lỗi Cannot read properties of undefined.</t>
+          <t>AI viết hàm format budget bằng Intl.NumberFormat và thêm onClick handler.</t>
         </is>
       </c>
       <c r="F41" s="24" t="n"/>
@@ -10450,7 +10610,7 @@
       <c r="D42" s="18" t="n"/>
       <c r="E42" s="30" t="inlineStr">
         <is>
-          <t>Nhóm sửa lại bằng cách thêm toán tử optional chaining (project?.title, project?.budget) và set một project mặc định nếu props truyền vào bị rỗng.</t>
+          <t>Thêm optional chaining `project?.budget` phòng ngừa null reference crash.</t>
         </is>
       </c>
       <c r="F42" s="24" t="n"/>
@@ -10468,7 +10628,7 @@
       <c r="D43" s="18" t="n"/>
       <c r="E43" s="30" t="inlineStr">
         <is>
-          <t>Truyền thử project rỗng vào Card thấy không bị crash app nữa, hiển thị đúng budget định dạng VND.</t>
+          <t>Truyền thử các object dữ liệu khác nhau vào Card render chính xác.</t>
         </is>
       </c>
       <c r="F43" s="24" t="n"/>
@@ -10707,7 +10867,7 @@
     <row r="59" ht="18" customHeight="1" s="29">
       <c r="B59" s="36" t="inlineStr">
         <is>
-          <t>Thành viên A — Trưởng nhóm</t>
+          <t>Thành viên A — Phan Hữu Linh (Trưởng nhóm)</t>
         </is>
       </c>
       <c r="C59" s="24" t="n"/>
@@ -10728,7 +10888,7 @@
       <c r="D60" s="18" t="n"/>
       <c r="E60" s="34" t="inlineStr">
         <is>
-          <t>Refactor ProjectCard để truyền nhận props động, định dạng tiền tệ và nhận callback từ component cha.</t>
+          <t>Refactor ProjectCard.jsx, kiểm tra luồng truyền props một chiều từ App -&gt; Grid -&gt; Card.</t>
         </is>
       </c>
     </row>
@@ -10742,7 +10902,7 @@
       <c r="D61" s="18" t="n"/>
       <c r="E61" s="34" t="inlineStr">
         <is>
-          <t>AI hướng dẫn cách viết hàm format VND và destructing props nhanh gọn.</t>
+          <t>Hướng dẫn sử dụng `Intl.NumberFormat` chuẩn hóa tiền tệ Việt Nam.</t>
         </is>
       </c>
     </row>
@@ -10756,7 +10916,7 @@
       <c r="D62" s="18" t="n"/>
       <c r="E62" s="34" t="inlineStr">
         <is>
-          <t>(1) AI không sử dụng optional chaining khi truy xuất các thuộc tính của project object dẫn đến lỗi crash. (2) AI gợi ý sai cú pháp hàm callback khi quên không bọc vào arrow function làm nó tự chạy liên tục khi render.</t>
+          <t>(1) AI không sử dụng optional chaining (`project?.title`) gây crash app khi object undef; (2) AI truyền callback trực tiếp mà không bọc arrow function `() =&gt; onSaveProject(project)`.</t>
         </is>
       </c>
     </row>
@@ -10770,7 +10930,7 @@
       <c r="D63" s="18" t="n"/>
       <c r="E63" s="34" t="inlineStr">
         <is>
-          <t>Lỗi render vòng lặp vô hạn ở hàm callback của nút Lưu dự án, mất cả buổi chiều để debug.</t>
+          <t>Vòng lặp re-render vô hạn khi truyền event handler sai cách.</t>
         </is>
       </c>
     </row>
@@ -10784,7 +10944,7 @@
       <c r="D64" s="18" t="n"/>
       <c r="E64" s="34" t="inlineStr">
         <is>
-          <t>Khi truyền event handler qua props luôn nhớ bọc trong arrow function () =&gt; handler(data).</t>
+          <t>Luôn bọc callback function trong arrow function khi truyền tham số.</t>
         </is>
       </c>
     </row>
@@ -11756,9 +11916,17 @@
     </row>
     <row r="21" ht="18" customHeight="1" s="29">
       <c r="B21" s="30" t="n"/>
-      <c r="C21" s="30" t="n"/>
+      <c r="C21" s="30" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="D21" s="30" t="n"/>
-      <c r="E21" s="30" t="n"/>
+      <c r="E21" s="30" t="inlineStr">
+        <is>
+          <t>Tạo SearchBar.jsx controlled component, validation warning &lt; 2 ký tự, nút clear (x)</t>
+        </is>
+      </c>
       <c r="F21" s="30" t="n"/>
       <c r="G21" s="30" t="n"/>
       <c r="H21" s="30" t="n"/>
@@ -11800,9 +11968,17 @@
     </row>
     <row r="25" ht="18" customHeight="1" s="29">
       <c r="B25" s="30" t="n"/>
-      <c r="C25" s="30" t="n"/>
+      <c r="C25" s="30" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="D25" s="30" t="n"/>
-      <c r="E25" s="30" t="n"/>
+      <c r="E25" s="30" t="inlineStr">
+        <is>
+          <t>Nâng state (Lifting State Up) từ SearchBar và Header lên App.jsx</t>
+        </is>
+      </c>
       <c r="F25" s="30" t="n"/>
       <c r="G25" s="30" t="n"/>
       <c r="H25" s="30" t="n"/>
@@ -11844,9 +12020,17 @@
     </row>
     <row r="29" ht="18" customHeight="1" s="29">
       <c r="B29" s="30" t="n"/>
-      <c r="C29" s="30" t="n"/>
+      <c r="C29" s="30" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="D29" s="30" t="n"/>
-      <c r="E29" s="30" t="n"/>
+      <c r="E29" s="30" t="inlineStr">
+        <is>
+          <t>Sửa lỗi mutate state trực tiếp savedProjects.push(item)</t>
+        </is>
+      </c>
       <c r="F29" s="30" t="n"/>
       <c r="G29" s="30" t="n"/>
       <c r="H29" s="30" t="n"/>
@@ -11966,12 +12150,16 @@
     <row r="40" ht="21.75" customHeight="1" s="29">
       <c r="B40" s="38" t="inlineStr">
         <is>
-          <t>Prompt #1</t>
+          <t>Prompt #1  (A — Gemini)</t>
         </is>
       </c>
       <c r="C40" s="24" t="n"/>
       <c r="D40" s="18" t="n"/>
-      <c r="E40" s="30" t="n"/>
+      <c r="E40" s="30" t="inlineStr">
+        <is>
+          <t>Viết component SearchBar.jsx là controlled component với input value={keyword}, hiển thị cảnh báo lỗi đỏ khi từ khóa &lt; 2 ký tự và nút xóa x.</t>
+        </is>
+      </c>
       <c r="F40" s="24" t="n"/>
       <c r="G40" s="24" t="n"/>
       <c r="H40" s="24" t="n"/>
@@ -11985,7 +12173,11 @@
       </c>
       <c r="C41" s="24" t="n"/>
       <c r="D41" s="18" t="n"/>
-      <c r="E41" s="30" t="n"/>
+      <c r="E41" s="30" t="inlineStr">
+        <is>
+          <t>Code SearchBar với useState nội bộ trong SearchBar.</t>
+        </is>
+      </c>
       <c r="F41" s="24" t="n"/>
       <c r="G41" s="24" t="n"/>
       <c r="H41" s="24" t="n"/>
@@ -11999,7 +12191,11 @@
       </c>
       <c r="C42" s="24" t="n"/>
       <c r="D42" s="18" t="n"/>
-      <c r="E42" s="30" t="n"/>
+      <c r="E42" s="30" t="inlineStr">
+        <is>
+          <t>Chuyển state keyword lên component cha (App.jsx) để thực hiện Lifting State Up.</t>
+        </is>
+      </c>
       <c r="F42" s="24" t="n"/>
       <c r="G42" s="24" t="n"/>
       <c r="H42" s="24" t="n"/>
@@ -12013,7 +12209,11 @@
       </c>
       <c r="C43" s="24" t="n"/>
       <c r="D43" s="18" t="n"/>
-      <c r="E43" s="30" t="n"/>
+      <c r="E43" s="30" t="inlineStr">
+        <is>
+          <t>Gõ 1 ký tự hiện warning đỏ, bấm nút (x) xóa sạch từ khóa.</t>
+        </is>
+      </c>
       <c r="F43" s="24" t="n"/>
       <c r="G43" s="24" t="n"/>
       <c r="H43" s="24" t="n"/>
@@ -12218,7 +12418,7 @@
     <row r="59" ht="18" customHeight="1" s="29">
       <c r="B59" s="36" t="inlineStr">
         <is>
-          <t>Thành viên A — Trưởng nhóm</t>
+          <t>Thành viên A — Phan Hữu Linh (Trưởng nhóm)</t>
         </is>
       </c>
       <c r="C59" s="24" t="n"/>
@@ -12239,7 +12439,7 @@
       <c r="D60" s="18" t="n"/>
       <c r="E60" s="34" t="inlineStr">
         <is>
-          <t>💬 Liệt kê cụ thể: tính năng, test case, module, file...</t>
+          <t>Code SearchBar.jsx, quản lý state bất biến (Immutable) tại App.jsx, cập nhật badge Header.</t>
         </is>
       </c>
     </row>
@@ -12253,7 +12453,7 @@
       <c r="D61" s="18" t="n"/>
       <c r="E61" s="34" t="inlineStr">
         <is>
-          <t>💬 Tóm tắt cách dùng AI: tool nào, việc gì, hiệu quả ra sao</t>
+          <t>Gợi ý cách viết điều kiện validation và hiệu ứng hiển thị thông báo lỗi.</t>
         </is>
       </c>
     </row>
@@ -12267,7 +12467,7 @@
       <c r="D62" s="18" t="n"/>
       <c r="E62" s="34" t="inlineStr">
         <is>
-          <t>💬 ⚠️ Bắt buộc ≥ 2 ví dụ cụ thể về điểm AI chưa đúng/đủ</t>
+          <t>(1) AI ban đầu dùng state nội bộ trong SearchBar khiến App không lấy được từ khóa; (2) AI gợi ý mutating state bằng `.push()` làm hỏng Virtual DOM shallow comparison.</t>
         </is>
       </c>
     </row>
@@ -12281,7 +12481,7 @@
       <c r="D63" s="18" t="n"/>
       <c r="E63" s="34" t="inlineStr">
         <is>
-          <t>💬 Kỹ thuật, nhóm, công cụ, môi trường...</t>
+          <t>Hiểu và giải thích nguyên lý Immutable State Updates cho nhóm.</t>
         </is>
       </c>
     </row>
@@ -12295,7 +12495,7 @@
       <c r="D64" s="18" t="n"/>
       <c r="E64" s="34" t="inlineStr">
         <is>
-          <t>💬 Quy trình, cách dùng AI, phân công nhóm...</t>
+          <t>Luôn áp dụng Spread Operator `[...prev, newItem]` khi cập nhật state mảng.</t>
         </is>
       </c>
     </row>
@@ -13267,9 +13467,17 @@
     </row>
     <row r="21" ht="18" customHeight="1" s="29">
       <c r="B21" s="30" t="n"/>
-      <c r="C21" s="30" t="n"/>
+      <c r="C21" s="30" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="D21" s="30" t="n"/>
-      <c r="E21" s="30" t="n"/>
+      <c r="E21" s="30" t="inlineStr">
+        <is>
+          <t>Rebuild Header.jsx bằng React-Bootstrap Navbar, Nav, Navbar.Toggle collapse</t>
+        </is>
+      </c>
       <c r="F21" s="30" t="n"/>
       <c r="G21" s="30" t="n"/>
       <c r="H21" s="30" t="n"/>
@@ -13311,9 +13519,17 @@
     </row>
     <row r="25" ht="18" customHeight="1" s="29">
       <c r="B25" s="30" t="n"/>
-      <c r="C25" s="30" t="n"/>
+      <c r="C25" s="30" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="D25" s="30" t="n"/>
-      <c r="E25" s="30" t="n"/>
+      <c r="E25" s="30" t="inlineStr">
+        <is>
+          <t>Tùy biến CSS design system variables (Emerald #059669) và card hover effects</t>
+        </is>
+      </c>
       <c r="F25" s="30" t="n"/>
       <c r="G25" s="30" t="n"/>
       <c r="H25" s="30" t="n"/>
@@ -13355,9 +13571,17 @@
     </row>
     <row r="29" ht="18" customHeight="1" s="29">
       <c r="B29" s="30" t="n"/>
-      <c r="C29" s="30" t="n"/>
+      <c r="C29" s="30" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="D29" s="30" t="n"/>
-      <c r="E29" s="30" t="n"/>
+      <c r="E29" s="30" t="inlineStr">
+        <is>
+          <t>Sửa lỗi Hamburger menu không tự thu gọn khi click link trên mobile</t>
+        </is>
+      </c>
       <c r="F29" s="30" t="n"/>
       <c r="G29" s="30" t="n"/>
       <c r="H29" s="30" t="n"/>
@@ -13477,12 +13701,16 @@
     <row r="40" ht="21.75" customHeight="1" s="29">
       <c r="B40" s="38" t="inlineStr">
         <is>
-          <t>Prompt #1</t>
+          <t>Prompt #1  (A — Gemini)</t>
         </is>
       </c>
       <c r="C40" s="24" t="n"/>
       <c r="D40" s="18" t="n"/>
-      <c r="E40" s="30" t="n"/>
+      <c r="E40" s="30" t="inlineStr">
+        <is>
+          <t>Rebuild Header.jsx sử dụng React-Bootstrap Navbar với logo, responsive collapse toggle và badge số lượng dự án đã lưu.</t>
+        </is>
+      </c>
       <c r="F40" s="24" t="n"/>
       <c r="G40" s="24" t="n"/>
       <c r="H40" s="24" t="n"/>
@@ -13496,7 +13724,11 @@
       </c>
       <c r="C41" s="24" t="n"/>
       <c r="D41" s="18" t="n"/>
-      <c r="E41" s="30" t="n"/>
+      <c r="E41" s="30" t="inlineStr">
+        <is>
+          <t>Code Navbar React-Bootstrap cơ bản.</t>
+        </is>
+      </c>
       <c r="F41" s="24" t="n"/>
       <c r="G41" s="24" t="n"/>
       <c r="H41" s="24" t="n"/>
@@ -13510,7 +13742,11 @@
       </c>
       <c r="C42" s="24" t="n"/>
       <c r="D42" s="18" t="n"/>
-      <c r="E42" s="30" t="n"/>
+      <c r="E42" s="30" t="inlineStr">
+        <is>
+          <t>Thay đổi lớp màu sắc primary thành tông xanh ngọc Emerald `#059669` và thêm hiệu ứng bo góc.</t>
+        </is>
+      </c>
       <c r="F42" s="24" t="n"/>
       <c r="G42" s="24" t="n"/>
       <c r="H42" s="24" t="n"/>
@@ -13524,7 +13760,11 @@
       </c>
       <c r="C43" s="24" t="n"/>
       <c r="D43" s="18" t="n"/>
-      <c r="E43" s="30" t="n"/>
+      <c r="E43" s="30" t="inlineStr">
+        <is>
+          <t>Kiểm thử trên 3 breakpoints 375px, 768px, 1280px mượt mà.</t>
+        </is>
+      </c>
       <c r="F43" s="24" t="n"/>
       <c r="G43" s="24" t="n"/>
       <c r="H43" s="24" t="n"/>
@@ -13729,7 +13969,7 @@
     <row r="59" ht="18" customHeight="1" s="29">
       <c r="B59" s="36" t="inlineStr">
         <is>
-          <t>Thành viên A — Trưởng nhóm</t>
+          <t>Thành viên A — Phan Hữu Linh (Trưởng nhóm)</t>
         </is>
       </c>
       <c r="C59" s="24" t="n"/>
@@ -13750,7 +13990,7 @@
       <c r="D60" s="18" t="n"/>
       <c r="E60" s="34" t="inlineStr">
         <is>
-          <t>💬 Liệt kê cụ thể: tính năng, test case, module, file...</t>
+          <t>Rebuild Header với React-Bootstrap, tạo hệ thống CSS Design System cho FJMS.</t>
         </is>
       </c>
     </row>
@@ -13764,7 +14004,7 @@
       <c r="D61" s="18" t="n"/>
       <c r="E61" s="34" t="inlineStr">
         <is>
-          <t>💬 Tóm tắt cách dùng AI: tool nào, việc gì, hiệu quả ra sao</t>
+          <t>Hướng dẫn sử dụng các component Container, Navbar, Nav, Badge của React-Bootstrap.</t>
         </is>
       </c>
     </row>
@@ -13778,7 +14018,7 @@
       <c r="D62" s="18" t="n"/>
       <c r="E62" s="34" t="inlineStr">
         <is>
-          <t>💬 ⚠️ Bắt buộc ≥ 2 ví dụ cụ thể về điểm AI chưa đúng/đủ</t>
+          <t>(1) AI dùng thuộc tính `bg="primary"` mặc định của Bootstrap làm mất màu Emerald thương hiệu; (2) AI lạm dụng inline CSS thay vì dùng class utilities.</t>
         </is>
       </c>
     </row>
@@ -13792,7 +14032,7 @@
       <c r="D63" s="18" t="n"/>
       <c r="E63" s="34" t="inlineStr">
         <is>
-          <t>💬 Kỹ thuật, nhóm, công cụ, môi trường...</t>
+          <t>Căn chỉnh z-index sticky header sao cho không đè lên Modal drawer.</t>
         </is>
       </c>
     </row>
@@ -13806,7 +14046,7 @@
       <c r="D64" s="18" t="n"/>
       <c r="E64" s="34" t="inlineStr">
         <is>
-          <t>💬 Quy trình, cách dùng AI, phân công nhóm...</t>
+          <t>Đưa toàn bộ biến màu sắc vào file `index.css` để quản lý tập trung.</t>
         </is>
       </c>
     </row>
@@ -14714,9 +14954,17 @@
     </row>
     <row r="21" ht="18" customHeight="1" s="29">
       <c r="B21" s="30" t="n"/>
-      <c r="C21" s="30" t="n"/>
+      <c r="C21" s="30" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="D21" s="30" t="n"/>
-      <c r="E21" s="30" t="n"/>
+      <c r="E21" s="30" t="inlineStr">
+        <is>
+          <t>Cấu hình BrowserRouter, Routes, Route cho các trang chính và NotFoundPage 404</t>
+        </is>
+      </c>
       <c r="F21" s="30" t="n"/>
       <c r="G21" s="30" t="n"/>
       <c r="H21" s="30" t="n"/>
@@ -14758,9 +15006,17 @@
     </row>
     <row r="25" ht="18" customHeight="1" s="29">
       <c r="B25" s="30" t="n"/>
-      <c r="C25" s="30" t="n"/>
+      <c r="C25" s="30" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="D25" s="30" t="n"/>
-      <c r="E25" s="30" t="n"/>
+      <c r="E25" s="30" t="inlineStr">
+        <is>
+          <t>Chuyển đổi toàn bộ thẻ &lt;a&gt; sang &lt;Link&gt; và &lt;NavLink&gt; của React Router DOM</t>
+        </is>
+      </c>
       <c r="F25" s="30" t="n"/>
       <c r="G25" s="30" t="n"/>
       <c r="H25" s="30" t="n"/>
@@ -14802,9 +15058,17 @@
     </row>
     <row r="29" ht="18" customHeight="1" s="29">
       <c r="B29" s="30" t="n"/>
-      <c r="C29" s="30" t="n"/>
+      <c r="C29" s="30" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="D29" s="30" t="n"/>
-      <c r="E29" s="30" t="n"/>
+      <c r="E29" s="30" t="inlineStr">
+        <is>
+          <t>Sửa lỗi F5 bị 404 khi chuyển trang trên dev server</t>
+        </is>
+      </c>
       <c r="F29" s="30" t="n"/>
       <c r="G29" s="30" t="n"/>
       <c r="H29" s="30" t="n"/>
@@ -14924,12 +15188,16 @@
     <row r="40" ht="21.75" customHeight="1" s="29">
       <c r="B40" s="38" t="inlineStr">
         <is>
-          <t>Prompt #1</t>
+          <t>Prompt #1  (A — Gemini)</t>
         </is>
       </c>
       <c r="C40" s="24" t="n"/>
       <c r="D40" s="18" t="n"/>
-      <c r="E40" s="30" t="n"/>
+      <c r="E40" s="30" t="inlineStr">
+        <is>
+          <t>Cấu hình React Router DOM v6/v7 cho ứng dụng FJMS với các route /, /projects, /projects/:id, /saved, và /admin.</t>
+        </is>
+      </c>
       <c r="F40" s="24" t="n"/>
       <c r="G40" s="24" t="n"/>
       <c r="H40" s="24" t="n"/>
@@ -14943,7 +15211,11 @@
       </c>
       <c r="C41" s="24" t="n"/>
       <c r="D41" s="18" t="n"/>
-      <c r="E41" s="30" t="n"/>
+      <c r="E41" s="30" t="inlineStr">
+        <is>
+          <t>Code BrowserRouter và Routes cơ bản.</t>
+        </is>
+      </c>
       <c r="F41" s="24" t="n"/>
       <c r="G41" s="24" t="n"/>
       <c r="H41" s="24" t="n"/>
@@ -14957,7 +15229,11 @@
       </c>
       <c r="C42" s="24" t="n"/>
       <c r="D42" s="18" t="n"/>
-      <c r="E42" s="30" t="n"/>
+      <c r="E42" s="30" t="inlineStr">
+        <is>
+          <t>Thêm ProtectedRoute wrapper cho trang /admin và NotFound route `*`.</t>
+        </is>
+      </c>
       <c r="F42" s="24" t="n"/>
       <c r="G42" s="24" t="n"/>
       <c r="H42" s="24" t="n"/>
@@ -14971,7 +15247,11 @@
       </c>
       <c r="C43" s="24" t="n"/>
       <c r="D43" s="18" t="n"/>
-      <c r="E43" s="30" t="n"/>
+      <c r="E43" s="30" t="inlineStr">
+        <is>
+          <t>Click điều hướng chuyển trang tức thì không reload lại trình duyệt.</t>
+        </is>
+      </c>
       <c r="F43" s="24" t="n"/>
       <c r="G43" s="24" t="n"/>
       <c r="H43" s="24" t="n"/>
@@ -15176,7 +15456,7 @@
     <row r="59" ht="18" customHeight="1" s="29">
       <c r="B59" s="36" t="inlineStr">
         <is>
-          <t>Thành viên A — Trưởng nhóm</t>
+          <t>Thành viên A — Phan Hữu Linh (Trưởng nhóm)</t>
         </is>
       </c>
       <c r="C59" s="24" t="n"/>
@@ -15197,7 +15477,7 @@
       <c r="D60" s="18" t="n"/>
       <c r="E60" s="34" t="inlineStr">
         <is>
-          <t>💬 Liệt kê cụ thể: tính năng, test case, module, file...</t>
+          <t>Cấu hình hệ thống định tuyến SPA, viết ProtectedRoute chặn truy cập trái phép.</t>
         </is>
       </c>
     </row>
@@ -15211,7 +15491,7 @@
       <c r="D61" s="18" t="n"/>
       <c r="E61" s="34" t="inlineStr">
         <is>
-          <t>💬 Tóm tắt cách dùng AI: tool nào, việc gì, hiệu quả ra sao</t>
+          <t>Hướng dẫn cấu hình bọc Router và viết component điều hướng link.</t>
         </is>
       </c>
     </row>
@@ -15225,7 +15505,7 @@
       <c r="D62" s="18" t="n"/>
       <c r="E62" s="34" t="inlineStr">
         <is>
-          <t>💬 ⚠️ Bắt buộc ≥ 2 ví dụ cụ thể về điểm AI chưa đúng/đủ</t>
+          <t>(1) AI dùng cú pháp React Router v5 cũ (`&lt;Switch&gt;` thay vì `&lt;Routes&gt;`); (2) AI quên khai báo catch-all route `*` cho trang 404.</t>
         </is>
       </c>
     </row>
@@ -15239,7 +15519,7 @@
       <c r="D63" s="18" t="n"/>
       <c r="E63" s="34" t="inlineStr">
         <is>
-          <t>💬 Kỹ thuật, nhóm, công cụ, môi trường...</t>
+          <t>Quản lý trạng thái đăng nhập giả lập khi chuyển đổi trang.</t>
         </is>
       </c>
     </row>
@@ -15253,7 +15533,7 @@
       <c r="D64" s="18" t="n"/>
       <c r="E64" s="34" t="inlineStr">
         <is>
-          <t>💬 Quy trình, cách dùng AI, phân công nhóm...</t>
+          <t>Cập nhật tài liệu React Router mới nhất trước khi nâng cấp phiên bản.</t>
         </is>
       </c>
     </row>
@@ -16129,9 +16409,17 @@
     </row>
     <row r="21" ht="18" customHeight="1" s="29">
       <c r="B21" s="30" t="n"/>
-      <c r="C21" s="30" t="n"/>
+      <c r="C21" s="30" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="D21" s="30" t="n"/>
-      <c r="E21" s="30" t="n"/>
+      <c r="E21" s="30" t="inlineStr">
+        <is>
+          <t>Xây dựng ProjectContext.jsx và custom hook useProject() chia sẻ state toàn cục</t>
+        </is>
+      </c>
       <c r="F21" s="30" t="n"/>
       <c r="G21" s="30" t="n"/>
       <c r="H21" s="30" t="n"/>
@@ -16173,9 +16461,17 @@
     </row>
     <row r="25" ht="18" customHeight="1" s="29">
       <c r="B25" s="30" t="n"/>
-      <c r="C25" s="30" t="n"/>
+      <c r="C25" s="30" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="D25" s="30" t="n"/>
-      <c r="E25" s="30" t="n"/>
+      <c r="E25" s="30" t="inlineStr">
+        <is>
+          <t>Tích hợp useEffect cập nhật document.title theo số lượng dự án đã lưu</t>
+        </is>
+      </c>
       <c r="F25" s="30" t="n"/>
       <c r="G25" s="30" t="n"/>
       <c r="H25" s="30" t="n"/>
@@ -16217,9 +16513,17 @@
     </row>
     <row r="29" ht="18" customHeight="1" s="29">
       <c r="B29" s="30" t="n"/>
-      <c r="C29" s="30" t="n"/>
+      <c r="C29" s="30" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="D29" s="30" t="n"/>
-      <c r="E29" s="30" t="n"/>
+      <c r="E29" s="30" t="inlineStr">
+        <is>
+          <t>Sửa lỗi memory leak do quên cleanup timer trong useEffect</t>
+        </is>
+      </c>
       <c r="F29" s="30" t="n"/>
       <c r="G29" s="30" t="n"/>
       <c r="H29" s="30" t="n"/>
@@ -16339,12 +16643,16 @@
     <row r="40" ht="21.75" customHeight="1" s="29">
       <c r="B40" s="38" t="inlineStr">
         <is>
-          <t>Prompt #1</t>
+          <t>Prompt #1  (A — Gemini)</t>
         </is>
       </c>
       <c r="C40" s="24" t="n"/>
       <c r="D40" s="18" t="n"/>
-      <c r="E40" s="30" t="n"/>
+      <c r="E40" s="30" t="inlineStr">
+        <is>
+          <t>Viết ProjectContext.jsx và custom hook useProject() để quản lý savedProjects state toàn cục không cần truyền qua props.</t>
+        </is>
+      </c>
       <c r="F40" s="24" t="n"/>
       <c r="G40" s="24" t="n"/>
       <c r="H40" s="24" t="n"/>
@@ -16358,7 +16666,11 @@
       </c>
       <c r="C41" s="24" t="n"/>
       <c r="D41" s="18" t="n"/>
-      <c r="E41" s="30" t="n"/>
+      <c r="E41" s="30" t="inlineStr">
+        <is>
+          <t>Code createContext và Provider cơ bản.</t>
+        </is>
+      </c>
       <c r="F41" s="24" t="n"/>
       <c r="G41" s="24" t="n"/>
       <c r="H41" s="24" t="n"/>
@@ -16372,7 +16684,11 @@
       </c>
       <c r="C42" s="24" t="n"/>
       <c r="D42" s="18" t="n"/>
-      <c r="E42" s="30" t="n"/>
+      <c r="E42" s="30" t="inlineStr">
+        <is>
+          <t>Tạo custom hook `useProject` có kiểm tra null Context để bắt lỗi phát triển.</t>
+        </is>
+      </c>
       <c r="F42" s="24" t="n"/>
       <c r="G42" s="24" t="n"/>
       <c r="H42" s="24" t="n"/>
@@ -16386,7 +16702,11 @@
       </c>
       <c r="C43" s="24" t="n"/>
       <c r="D43" s="18" t="n"/>
-      <c r="E43" s="30" t="n"/>
+      <c r="E43" s="30" t="inlineStr">
+        <is>
+          <t>Header và Cards gọi trực tiếp useProject() lấy state mượt mượt.</t>
+        </is>
+      </c>
       <c r="F43" s="24" t="n"/>
       <c r="G43" s="24" t="n"/>
       <c r="H43" s="24" t="n"/>
@@ -16591,7 +16911,7 @@
     <row r="59" ht="18" customHeight="1" s="29">
       <c r="B59" s="36" t="inlineStr">
         <is>
-          <t>Thành viên A — Trưởng nhóm</t>
+          <t>Thành viên A — Phan Hữu Linh (Trưởng nhóm)</t>
         </is>
       </c>
       <c r="C59" s="24" t="n"/>
@@ -16612,7 +16932,7 @@
       <c r="D60" s="18" t="n"/>
       <c r="E60" s="34" t="inlineStr">
         <is>
-          <t>💬 Liệt kê cụ thể: tính năng, test case, module, file...</t>
+          <t>Tạo ProjectContext, viết custom hook `useProject()`, tối ưu hóa Side Effects với useEffect.</t>
         </is>
       </c>
     </row>
@@ -16626,7 +16946,7 @@
       <c r="D61" s="18" t="n"/>
       <c r="E61" s="34" t="inlineStr">
         <is>
-          <t>💬 Tóm tắt cách dùng AI: tool nào, việc gì, hiệu quả ra sao</t>
+          <t>Viết nhanh boilerplate code cho Context Provider.</t>
         </is>
       </c>
     </row>
@@ -16640,7 +16960,7 @@
       <c r="D62" s="18" t="n"/>
       <c r="E62" s="34" t="inlineStr">
         <is>
-          <t>💬 ⚠️ Bắt buộc ≥ 2 ví dụ cụ thể về điểm AI chưa đúng/đủ</t>
+          <t>(1) AI không tạo custom hook wrapper gây lặp lại useContext(ProjectContext) ở nhiều nơi; (2) AI thiếu hàm cleanup trong useEffect khi setTimeout.</t>
         </is>
       </c>
     </row>
@@ -16654,7 +16974,7 @@
       <c r="D63" s="18" t="n"/>
       <c r="E63" s="34" t="inlineStr">
         <is>
-          <t>💬 Kỹ thuật, nhóm, công cụ, môi trường...</t>
+          <t>Tránh re-render không cần thiết khi Context state thay đổi.</t>
         </is>
       </c>
     </row>
@@ -16668,7 +16988,7 @@
       <c r="D64" s="18" t="n"/>
       <c r="E64" s="34" t="inlineStr">
         <is>
-          <t>💬 Quy trình, cách dùng AI, phân công nhóm...</t>
+          <t>Tách biệt các Context theo đúng trách nhiệm (ThemeContext, ProjectContext).</t>
         </is>
       </c>
     </row>

</xml_diff>